<commit_message>
fix: corrige tablas y disponibilidad de envío
Ajusta Table 3 y las tablas anchas del suplemento para que sean legibles en DOCX, repara los epígrafes de los maestros y sincroniza la disponibilidad de datos v2.0.1, el release v2.1.0 y el contenido S1–S11.
</commit_message>
<xml_diff>
--- a/entregables/tablas_maestro.xlsx
+++ b/entregables/tablas_maestro.xlsx
@@ -1156,7 +1156,7 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Cost-loss values by region, task, model and , with 95 % date-grouped bootstrap intervals (B = 1 000). FWI and INPE rows use their frozen F0.5 cutoffs (3.1285/20.4720 and 0.0364/0.0596, Chaco/Oriental); model rows use . is clipped at −1; the frozen FWI/INPE rows reach this bound for .</t>
+          <t>Cost-loss values by region, task, model and α, with 95 % date-grouped bootstrap intervals (B = 1 000). FWI and INPE rows use their frozen F0.5 cutoffs (3.1285/20.4720 and 0.0364/0.0596, Chaco/Oriental); model rows use p≥α. V is clipped at −1; the frozen FWI/INPE rows reach this bound for α≥0.001.</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -8031,7 +8031,7 @@
     <row r="1" ht="42" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Table S14. Cost-loss values by region, task, model and , with 95 % date-grouped bootstrap intervals (B = 1 000). FWI and INPE rows use their frozen F0.5 cutoffs (3.1285/20.4720 and 0.0364/0.0596, Chaco/Oriental); model rows use . is clipped at −1; the frozen FWI/INPE rows reach this bound for .</t>
+          <t>Table S14. Cost-loss values by region, task, model and α, with 95 % date-grouped bootstrap intervals (B = 1 000). FWI and INPE rows use their frozen F0.5 cutoffs (3.1285/20.4720 and 0.0364/0.0596, Chaco/Oriental); model rows use p≥α. V is clipped at −1; the frozen FWI/INPE rows reach this bound for α≥0.001.</t>
         </is>
       </c>
     </row>
@@ -34218,7 +34218,7 @@
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -34256,7 +34256,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>ΔROC (M3 − reference)</t>
+          <t>ΔROC</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">

</xml_diff>